<commit_message>
testing integration if using dt in numerator only
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{142521C7-6124-4DB2-BEC1-975610FAE575}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95555E3E-4239-4EA8-B1E7-1CBBC2610AE4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="948" windowWidth="21600" windowHeight="11292" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
     <sheet name="GM_BE_H2_CO2_T32_P1500" sheetId="17" r:id="rId10"/>
+    <sheet name="GM2_BE_H2CO2_T32_P1500_2" sheetId="18" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="24">
   <si>
     <t>KL/D0</t>
   </si>
@@ -115,6 +116,9 @@
   <si>
     <t>GomezMendez_etal_2026</t>
   </si>
+  <si>
+    <t>GGomezMendez_etal_2026</t>
+  </si>
 </sst>
 </file>
 
@@ -166,6 +170,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -900,6 +908,161 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD6862D5-821E-4960-8A9A-342FC0727C42}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.40720000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.255637</v>
+      </c>
+      <c r="B13">
+        <v>0.65700000000000003</v>
+      </c>
+      <c r="C13">
+        <f>B13/$B$9</f>
+        <v>1.6134577603143418</v>
+      </c>
+      <c r="D13">
+        <f>$B$7*A13/$B$9</f>
+        <v>0.84124160117878199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.51127500000000003</v>
+      </c>
+      <c r="B14">
+        <v>1.0037</v>
+      </c>
+      <c r="C14">
+        <f>B14/$B$9</f>
+        <v>2.4648821218074657</v>
+      </c>
+      <c r="D14">
+        <f>$B$7*A14/$B$9</f>
+        <v>1.6824864931237724</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.2781899000000001</v>
+      </c>
+      <c r="B15">
+        <v>1.5210999999999999</v>
+      </c>
+      <c r="C15">
+        <f>B15/$B$9</f>
+        <v>3.735510805500982</v>
+      </c>
+      <c r="D15">
+        <f>$B$7*A15/$B$9</f>
+        <v>4.2062241306483301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA757B11-61BA-4343-990A-779EA69AE742}">
   <dimension ref="A1:D25"/>
@@ -3266,4 +3429,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7cf48d45-3ddb-4389-a9c1-c115526eb52e}" enabled="0" method="" siteId="{7cf48d45-3ddb-4389-a9c1-c115526eb52e}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
fitting with Llines fixed, and vlines fixed dt varied to have Llines fixed, fitting in all C ranges from 0 to 100 %, more error but tortuosity and alpha with sense
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="338" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95555E3E-4239-4EA8-B1E7-1CBBC2610AE4}"/>
+  <xr:revisionPtr revIDLastSave="351" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AF1CF5F-F050-4286-8E2E-0C18C41E92CB}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="948" windowWidth="21600" windowHeight="11292" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18560" yWindow="640" windowWidth="14400" windowHeight="7350" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,9 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
     <sheet name="GM_BE_H2_CO2_T32_P1500" sheetId="17" r:id="rId10"/>
-    <sheet name="GM2_BE_H2CO2_T32_P1500_2" sheetId="18" r:id="rId11"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_2" sheetId="18" r:id="rId11"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_3" sheetId="19" r:id="rId12"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_4" sheetId="20" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="26">
   <si>
     <t>KL/D0</t>
   </si>
@@ -118,6 +120,12 @@
   </si>
   <si>
     <t>GGomezMendez_etal_2026</t>
+  </si>
+  <si>
+    <t>GGGomezMendez_etal_2026</t>
+  </si>
+  <si>
+    <t>GGGGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -1063,6 +1071,316 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03768FF1-13C5-49B9-B8B0-FBC9D51F7DEE}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.40720000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.255637</v>
+      </c>
+      <c r="B13">
+        <v>0.622</v>
+      </c>
+      <c r="C13">
+        <f>B13/$B$9</f>
+        <v>1.5275049115913555</v>
+      </c>
+      <c r="D13">
+        <f>$B$7*A13/$B$9</f>
+        <v>0.84124160117878199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.51127500000000003</v>
+      </c>
+      <c r="B14">
+        <v>0.98650000000000004</v>
+      </c>
+      <c r="C14">
+        <f>B14/$B$9</f>
+        <v>2.4226424361493124</v>
+      </c>
+      <c r="D14">
+        <f>$B$7*A14/$B$9</f>
+        <v>1.6824864931237724</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.2781899000000001</v>
+      </c>
+      <c r="B15">
+        <v>1.5989</v>
+      </c>
+      <c r="C15">
+        <f>B15/$B$9</f>
+        <v>3.9265717092337917</v>
+      </c>
+      <c r="D15">
+        <f>$B$7*A15/$B$9</f>
+        <v>4.2062241306483301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D8EE9D-5235-450B-97D3-5ED504571A13}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.40720000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.255637</v>
+      </c>
+      <c r="B13">
+        <v>0.60670000000000002</v>
+      </c>
+      <c r="C13">
+        <f>B13/$B$9</f>
+        <v>1.4899312377210217</v>
+      </c>
+      <c r="D13">
+        <f>$B$7*A13/$B$9</f>
+        <v>0.84124160117878199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.51127500000000003</v>
+      </c>
+      <c r="B14">
+        <v>1.1341000000000001</v>
+      </c>
+      <c r="C14">
+        <f>B14/$B$9</f>
+        <v>2.7851178781925348</v>
+      </c>
+      <c r="D14">
+        <f>$B$7*A14/$B$9</f>
+        <v>1.6824864931237724</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.2781899000000001</v>
+      </c>
+      <c r="B15">
+        <v>1.9715</v>
+      </c>
+      <c r="C15">
+        <f>B15/$B$9</f>
+        <v>4.8416011787819251</v>
+      </c>
+      <c r="D15">
+        <f>$B$7*A15/$B$9</f>
+        <v>4.2062241306483301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA757B11-61BA-4343-990A-779EA69AE742}">
   <dimension ref="A1:D25"/>

</xml_diff>

<commit_message>
processing2 with residuals and nlinfit with jacobian and such
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="351" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AF1CF5F-F050-4286-8E2E-0C18C41E92CB}"/>
+  <xr:revisionPtr revIDLastSave="359" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9572DDB-114A-4D20-82FB-77B545E016D8}"/>
   <bookViews>
-    <workbookView xWindow="-18560" yWindow="640" windowWidth="14400" windowHeight="7350" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="GM_BE_H2CO2_T32_P1500_2" sheetId="18" r:id="rId11"/>
     <sheet name="GM_BE_H2CO2_T32_P1500_3" sheetId="19" r:id="rId12"/>
     <sheet name="GM_BE_H2CO2_T32_P1500_4" sheetId="20" r:id="rId13"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="27">
   <si>
     <t>KL/D0</t>
   </si>
@@ -126,6 +127,9 @@
   </si>
   <si>
     <t>GGGGomezMendez_etal_2026</t>
+  </si>
+  <si>
+    <t>GGGGGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -1381,6 +1385,161 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A19B645C-29D5-4CC1-AB25-EDCCDCB6D159}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.40720000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.255637</v>
+      </c>
+      <c r="B13">
+        <v>0.58760000000000001</v>
+      </c>
+      <c r="C13">
+        <f>B13/$B$9</f>
+        <v>1.4430255402750491</v>
+      </c>
+      <c r="D13">
+        <f>$B$7*A13/$B$9</f>
+        <v>0.48967794695481337</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.51127500000000003</v>
+      </c>
+      <c r="B14">
+        <v>0.80469999999999997</v>
+      </c>
+      <c r="C14">
+        <f>B14/$B$9</f>
+        <v>1.9761787819253438</v>
+      </c>
+      <c r="D14">
+        <f>$B$7*A14/$B$9</f>
+        <v>0.97935780943025552</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.2781899000000001</v>
+      </c>
+      <c r="B15">
+        <v>1.3879999999999999</v>
+      </c>
+      <c r="C15">
+        <f>B15/$B$9</f>
+        <v>3.4086444007858545</v>
+      </c>
+      <c r="D15">
+        <f>$B$7*A15/$B$9</f>
+        <v>2.4483991208251474</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA757B11-61BA-4343-990A-779EA69AE742}">
   <dimension ref="A1:D25"/>

</xml_diff>

<commit_message>
fitting alpha tortuosity and beta with different models and constrains
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="359" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9572DDB-114A-4D20-82FB-77B545E016D8}"/>
+  <xr:revisionPtr revIDLastSave="364" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40166CC5-A419-412D-A55E-F96358CF6379}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -22,11 +22,7 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P1088" sheetId="8" r:id="rId7"/>
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
-    <sheet name="GM_BE_H2_CO2_T32_P1500" sheetId="17" r:id="rId10"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_2" sheetId="18" r:id="rId11"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_3" sheetId="19" r:id="rId12"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_4" sheetId="20" r:id="rId13"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId14"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="23">
   <si>
     <t>KL/D0</t>
   </si>
@@ -118,18 +114,6 @@
   </si>
   <si>
     <t>GomezMendez_etal_2026</t>
-  </si>
-  <si>
-    <t>GGomezMendez_etal_2026</t>
-  </si>
-  <si>
-    <t>GGGomezMendez_etal_2026</t>
-  </si>
-  <si>
-    <t>GGGGomezMendez_etal_2026</t>
-  </si>
-  <si>
-    <t>GGGGGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -766,626 +750,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C465F19A-C77A-433E-B732-B5F1D3D2B978}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0.193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>2.0499999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>0.40720000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.255637</v>
-      </c>
-      <c r="B13">
-        <v>0.90585499999999997</v>
-      </c>
-      <c r="C13">
-        <f>B13/$B$9</f>
-        <v>2.2245947937131629</v>
-      </c>
-      <c r="D13">
-        <f>$B$7*A13/$B$9</f>
-        <v>1.2869740913555991</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.51127500000000003</v>
-      </c>
-      <c r="B14">
-        <v>1.7183516299999999</v>
-      </c>
-      <c r="C14">
-        <f>B14/$B$9</f>
-        <v>4.2199205058939091</v>
-      </c>
-      <c r="D14">
-        <f>$B$7*A14/$B$9</f>
-        <v>2.5739532170923378</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1.2781899000000001</v>
-      </c>
-      <c r="B15">
-        <v>3.0809527999999999</v>
-      </c>
-      <c r="C15">
-        <f>B15/$B$9</f>
-        <v>7.566190569744597</v>
-      </c>
-      <c r="D15">
-        <f>$B$7*A15/$B$9</f>
-        <v>6.4348951252455793</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD6862D5-821E-4960-8A9A-342FC0727C42}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0.193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>1.34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>0.40720000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.255637</v>
-      </c>
-      <c r="B13">
-        <v>0.65700000000000003</v>
-      </c>
-      <c r="C13">
-        <f>B13/$B$9</f>
-        <v>1.6134577603143418</v>
-      </c>
-      <c r="D13">
-        <f>$B$7*A13/$B$9</f>
-        <v>0.84124160117878199</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.51127500000000003</v>
-      </c>
-      <c r="B14">
-        <v>1.0037</v>
-      </c>
-      <c r="C14">
-        <f>B14/$B$9</f>
-        <v>2.4648821218074657</v>
-      </c>
-      <c r="D14">
-        <f>$B$7*A14/$B$9</f>
-        <v>1.6824864931237724</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1.2781899000000001</v>
-      </c>
-      <c r="B15">
-        <v>1.5210999999999999</v>
-      </c>
-      <c r="C15">
-        <f>B15/$B$9</f>
-        <v>3.735510805500982</v>
-      </c>
-      <c r="D15">
-        <f>$B$7*A15/$B$9</f>
-        <v>4.2062241306483301</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03768FF1-13C5-49B9-B8B0-FBC9D51F7DEE}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0.193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>1.34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>0.40720000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.255637</v>
-      </c>
-      <c r="B13">
-        <v>0.622</v>
-      </c>
-      <c r="C13">
-        <f>B13/$B$9</f>
-        <v>1.5275049115913555</v>
-      </c>
-      <c r="D13">
-        <f>$B$7*A13/$B$9</f>
-        <v>0.84124160117878199</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.51127500000000003</v>
-      </c>
-      <c r="B14">
-        <v>0.98650000000000004</v>
-      </c>
-      <c r="C14">
-        <f>B14/$B$9</f>
-        <v>2.4226424361493124</v>
-      </c>
-      <c r="D14">
-        <f>$B$7*A14/$B$9</f>
-        <v>1.6824864931237724</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1.2781899000000001</v>
-      </c>
-      <c r="B15">
-        <v>1.5989</v>
-      </c>
-      <c r="C15">
-        <f>B15/$B$9</f>
-        <v>3.9265717092337917</v>
-      </c>
-      <c r="D15">
-        <f>$B$7*A15/$B$9</f>
-        <v>4.2062241306483301</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23D8EE9D-5235-450B-97D3-5ED504571A13}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0.193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>1.34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>0.40720000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.255637</v>
-      </c>
-      <c r="B13">
-        <v>0.60670000000000002</v>
-      </c>
-      <c r="C13">
-        <f>B13/$B$9</f>
-        <v>1.4899312377210217</v>
-      </c>
-      <c r="D13">
-        <f>$B$7*A13/$B$9</f>
-        <v>0.84124160117878199</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.51127500000000003</v>
-      </c>
-      <c r="B14">
-        <v>1.1341000000000001</v>
-      </c>
-      <c r="C14">
-        <f>B14/$B$9</f>
-        <v>2.7851178781925348</v>
-      </c>
-      <c r="D14">
-        <f>$B$7*A14/$B$9</f>
-        <v>1.6824864931237724</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1.2781899000000001</v>
-      </c>
-      <c r="B15">
-        <v>1.9715</v>
-      </c>
-      <c r="C15">
-        <f>B15/$B$9</f>
-        <v>4.8416011787819251</v>
-      </c>
-      <c r="D15">
-        <f>$B$7*A15/$B$9</f>
-        <v>4.2062241306483301</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A19B645C-29D5-4CC1-AB25-EDCCDCB6D159}">
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1398,7 +762,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
results for paper no tortuosity yes integration, alpha and KL with sensitivity analysis
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="364" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40166CC5-A419-412D-A55E-F96358CF6379}"/>
+  <xr:revisionPtr revIDLastSave="368" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1BC1358-6400-4665-85E3-F9353679A3E0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -166,10 +166,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -436,13 +432,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -450,7 +446,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -458,7 +454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -466,7 +462,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -474,7 +470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -482,7 +478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -490,7 +486,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -498,7 +494,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -506,7 +502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -514,7 +510,7 @@
         <v>0.435</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -528,7 +524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -536,7 +532,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -552,7 +548,7 @@
         <v>1.9236781609195404</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -568,7 +564,7 @@
         <v>1.7312643678160919</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -584,7 +580,7 @@
         <v>1.5390804597701151</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -600,7 +596,7 @@
         <v>1.3466666666666667</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -616,7 +612,7 @@
         <v>1.1542528735632185</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -632,7 +628,7 @@
         <v>0.96183908045977018</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -648,7 +644,7 @@
         <v>0.76942528735632187</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -664,7 +660,7 @@
         <v>0.57701149425287357</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -680,7 +676,7 @@
         <v>0.38482758620689655</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -696,7 +692,7 @@
         <v>0.19241379310344828</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -712,7 +708,7 @@
         <v>0.14436781609195404</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -728,7 +724,7 @@
         <v>9.6091954022988521E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -752,12 +748,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A19B645C-29D5-4CC1-AB25-EDCCDCB6D159}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -765,7 +761,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -773,7 +769,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -781,7 +777,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -789,7 +785,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -797,7 +793,7 @@
         <v>15.25</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -805,15 +801,15 @@
         <v>0.193</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+        <v>2.6150000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -821,7 +817,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -829,7 +825,7 @@
         <v>0.40720000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -843,7 +839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -851,52 +847,52 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>0.255637</v>
       </c>
       <c r="B13">
-        <v>0.58760000000000001</v>
+        <v>1.0456000000000001</v>
       </c>
       <c r="C13">
         <f>B13/$B$9</f>
-        <v>1.4430255402750491</v>
+        <v>2.5677799607072691</v>
       </c>
       <c r="D13">
         <f>$B$7*A13/$B$9</f>
-        <v>0.48967794695481337</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1.6416767067779963</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0.51127500000000003</v>
       </c>
       <c r="B14">
-        <v>0.80469999999999997</v>
+        <v>1.4628000000000001</v>
       </c>
       <c r="C14">
         <f>B14/$B$9</f>
-        <v>1.9761787819253438</v>
+        <v>3.5923379174852652</v>
       </c>
       <c r="D14">
         <f>$B$7*A14/$B$9</f>
-        <v>0.97935780943025552</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>3.2833598354616904</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1.2781899000000001</v>
       </c>
       <c r="B15">
-        <v>1.3879999999999999</v>
+        <v>2.4708999999999999</v>
       </c>
       <c r="C15">
         <f>B15/$B$9</f>
-        <v>3.4086444007858545</v>
+        <v>6.0680255402750491</v>
       </c>
       <c r="D15">
         <f>$B$7*A15/$B$9</f>
-        <v>2.4483991208251474</v>
+        <v>8.2084150012279</v>
       </c>
     </row>
   </sheetData>
@@ -907,13 +903,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA757B11-61BA-4343-990A-779EA69AE742}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -921,7 +917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -929,7 +925,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -937,7 +933,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -945,7 +941,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -953,7 +949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -961,7 +957,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -969,7 +965,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -977,7 +973,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -985,7 +981,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -999,7 +995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1007,7 +1003,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7.5309999999999997</v>
       </c>
@@ -1023,7 +1019,7 @@
         <v>1.298448275862069</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>6.6950000000000003</v>
       </c>
@@ -1039,7 +1035,7 @@
         <v>1.1543103448275864</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>5.8579999999999997</v>
       </c>
@@ -1055,7 +1051,7 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.0209999999999999</v>
       </c>
@@ -1071,7 +1067,7 @@
         <v>0.86568965517241381</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>4.1840000000000002</v>
       </c>
@@ -1087,7 +1083,7 @@
         <v>0.72137931034482772</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3.347</v>
       </c>
@@ -1103,7 +1099,7 @@
         <v>0.57706896551724141</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2.5099999999999998</v>
       </c>
@@ -1119,7 +1115,7 @@
         <v>0.4327586206896552</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -1135,7 +1131,7 @@
         <v>0.2886206896551724</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>0.83699999999999997</v>
       </c>
@@ -1151,7 +1147,7 @@
         <v>0.1443103448275862</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.628</v>
       </c>
@@ -1167,7 +1163,7 @@
         <v>0.10827586206896554</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.41799999999999998</v>
       </c>
@@ -1183,7 +1179,7 @@
         <v>7.2068965517241387E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.20899999999999999</v>
       </c>
@@ -1199,7 +1195,7 @@
         <v>3.6034482758620694E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2.0920000000000001</v>
       </c>
@@ -1223,13 +1219,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4622695-DEB5-4C1F-9455-6739E3C55888}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1237,7 +1233,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1245,7 +1241,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1253,7 +1249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1261,7 +1257,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1269,7 +1265,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1277,7 +1273,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1285,7 +1281,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1293,7 +1289,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1301,7 +1297,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1315,7 +1311,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1323,7 +1319,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5.8579999999999997</v>
       </c>
@@ -1339,7 +1335,7 @@
         <v>0.67333333333333334</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5.0209999999999999</v>
       </c>
@@ -1355,7 +1351,7 @@
         <v>0.57712643678160924</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4.1840000000000002</v>
       </c>
@@ -1371,7 +1367,7 @@
         <v>0.48091954022988509</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>3.347</v>
       </c>
@@ -1387,7 +1383,7 @@
         <v>0.38471264367816094</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2.9289999999999998</v>
       </c>
@@ -1403,7 +1399,7 @@
         <v>0.33666666666666667</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2.5099999999999998</v>
       </c>
@@ -1419,7 +1415,7 @@
         <v>0.28850574712643678</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2.0920000000000001</v>
       </c>
@@ -1435,7 +1431,7 @@
         <v>0.24045977011494254</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -1451,7 +1447,7 @@
         <v>0.19241379310344828</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.2549999999999999</v>
       </c>
@@ -1467,7 +1463,7 @@
         <v>0.14425287356321839</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -1483,7 +1479,7 @@
         <v>9.6206896551724139E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -1499,7 +1495,7 @@
         <v>7.2183908045977019E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -1515,7 +1511,7 @@
         <v>4.8045977011494261E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -1539,13 +1535,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F522CD30-DFF9-46D4-B41C-E2D69E5568A2}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1553,7 +1549,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1561,7 +1557,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1569,7 +1565,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1577,7 +1573,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1585,7 +1581,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1593,7 +1589,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1601,7 +1597,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1609,7 +1605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1617,7 +1613,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1631,7 +1627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1639,7 +1635,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -1655,7 +1651,7 @@
         <v>1.8112554112554113</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -1671,7 +1667,7 @@
         <v>1.63008658008658</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -1687,7 +1683,7 @@
         <v>1.4491341991341993</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -1703,7 +1699,7 @@
         <v>1.267965367965368</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -1719,7 +1715,7 @@
         <v>1.0867965367965366</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -1735,7 +1731,7 @@
         <v>0.90562770562770567</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -1751,7 +1747,7 @@
         <v>0.72445887445887447</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -1767,7 +1763,7 @@
         <v>0.54329004329004327</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -1783,7 +1779,7 @@
         <v>0.36233766233766229</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -1799,7 +1795,7 @@
         <v>0.18116883116883115</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -1815,7 +1811,7 @@
         <v>0.13593073593073593</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -1831,7 +1827,7 @@
         <v>9.0476190476190474E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -1855,13 +1851,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3833D965-A191-44EF-B626-D5738955DDF0}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1869,7 +1865,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1877,7 +1873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1885,7 +1881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1893,7 +1889,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1901,7 +1897,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1909,7 +1905,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1917,7 +1913,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1925,7 +1921,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1933,7 +1929,7 @@
         <v>0.61599999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1947,7 +1943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1955,7 +1951,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -1971,7 +1967,7 @@
         <v>1.3584415584415586</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -1987,7 +1983,7 @@
         <v>1.222564935064935</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -2003,7 +1999,7 @@
         <v>1.0868506493506496</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2019,7 +2015,7 @@
         <v>0.95097402597402592</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -2035,7 +2031,7 @@
         <v>0.8150974025974026</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -2051,7 +2047,7 @@
         <v>0.67922077922077928</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -2067,7 +2063,7 @@
         <v>0.54334415584415585</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -2083,7 +2079,7 @@
         <v>0.40746753246753248</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -2099,7 +2095,7 @@
         <v>0.27175324675324675</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -2115,7 +2111,7 @@
         <v>0.13587662337662337</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -2131,7 +2127,7 @@
         <v>0.10194805194805197</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -2147,7 +2143,7 @@
         <v>6.7857142857142866E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -2171,13 +2167,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C470E87-970C-4464-80DC-21CD570DB714}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2185,7 +2181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2193,7 +2189,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2201,7 +2197,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2209,7 +2205,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2217,7 +2213,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2225,7 +2221,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2233,7 +2229,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2241,7 +2237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2249,7 +2245,7 @@
         <v>0.92400000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2263,7 +2259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2271,7 +2267,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -2287,7 +2283,7 @@
         <v>0.90562770562770567</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -2303,7 +2299,7 @@
         <v>0.81504329004329001</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -2319,7 +2315,7 @@
         <v>0.72456709956709964</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2335,7 +2331,7 @@
         <v>0.63398268398268398</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -2351,7 +2347,7 @@
         <v>0.54339826839826832</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -2367,7 +2363,7 @@
         <v>0.45281385281385284</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -2383,7 +2379,7 @@
         <v>0.36222943722943723</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -2399,7 +2395,7 @@
         <v>0.27164502164502163</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -2415,7 +2411,7 @@
         <v>0.18116883116883115</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -2431,7 +2427,7 @@
         <v>9.0584415584415573E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -2447,7 +2443,7 @@
         <v>6.7965367965367965E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -2463,7 +2459,7 @@
         <v>4.5238095238095237E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -2487,13 +2483,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC97105-E75A-4887-9BED-937003238E58}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2501,7 +2497,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2509,7 +2505,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2517,7 +2513,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2525,7 +2521,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2533,7 +2529,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2537,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2549,7 +2545,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2557,7 +2553,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2565,7 +2561,7 @@
         <v>0.51200000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2579,7 +2575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2587,7 +2583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1.85</v>
       </c>
@@ -2603,7 +2599,7 @@
         <v>0.36132812500000006</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3</v>
       </c>
@@ -2619,7 +2615,7 @@
         <v>0.58593750000000011</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4.25</v>
       </c>
@@ -2643,13 +2639,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EB6648-E8BE-46BE-A305-6B6827CCA731}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2657,7 +2653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2665,7 +2661,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2673,7 +2669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2681,7 +2677,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2689,7 +2685,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2697,7 +2693,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2705,7 +2701,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2713,7 +2709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2721,7 +2717,7 @@
         <v>0.76800000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2735,7 +2731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2743,7 +2739,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -2759,7 +2755,7 @@
         <v>1.0895833333333333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -2775,7 +2771,7 @@
         <v>0.98059895833333333</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -2791,7 +2787,7 @@
         <v>0.87174479166666674</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2807,7 +2803,7 @@
         <v>0.76276041666666661</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>4.1840000000000002</v>
       </c>
@@ -2823,7 +2819,7 @@
         <v>0.54479166666666667</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>3.347</v>
       </c>
@@ -2839,7 +2835,7 @@
         <v>0.43580729166666665</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2.5099999999999998</v>
       </c>
@@ -2855,7 +2851,7 @@
         <v>0.32682291666666669</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -2871,7 +2867,7 @@
         <v>0.21796874999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>0.83699999999999997</v>
       </c>
@@ -2887,7 +2883,7 @@
         <v>0.10898437499999999</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.628</v>
       </c>
@@ -2903,7 +2899,7 @@
         <v>8.1770833333333348E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.41799999999999998</v>
       </c>
@@ -2919,7 +2915,7 @@
         <v>5.4427083333333334E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.20899999999999999</v>
       </c>
@@ -2943,13 +2939,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316B93C2-C5E9-456C-B87A-12E89A2041DB}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="4" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2957,7 +2953,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2965,7 +2961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2973,7 +2969,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2981,7 +2977,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2989,7 +2985,7 @@
         <v>10.130000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2997,7 +2993,7 @@
         <v>0.20799999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3005,7 +3001,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -3013,7 +3009,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -3021,7 +3017,7 @@
         <v>0.92400000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -3035,7 +3031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -3043,7 +3039,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7.22</v>
       </c>
@@ -3059,7 +3055,7 @@
         <v>0.24222943722943721</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5.7799999999999994</v>
       </c>
@@ -3075,7 +3071,7 @@
         <v>0.19391774891774888</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4.33</v>
       </c>
@@ -3091,7 +3087,7 @@
         <v>0.14527056277056274</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>3.61</v>
       </c>
@@ -3107,7 +3103,7 @@
         <v>0.12111471861471861</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2.89</v>
       </c>
@@ -3123,7 +3119,7 @@
         <v>9.6958874458874453E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2.17</v>
       </c>
@@ -3139,7 +3135,7 @@
         <v>7.28030303030303E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1.81</v>
       </c>
@@ -3155,7 +3151,7 @@
         <v>6.0725108225108224E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1.44</v>
       </c>
@@ -3171,7 +3167,7 @@
         <v>4.8311688311688306E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1.08</v>
       </c>
@@ -3187,7 +3183,7 @@
         <v>3.6233766233766236E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>0.72</v>
       </c>
@@ -3203,7 +3199,7 @@
         <v>2.4155844155844153E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>0.54</v>
       </c>
@@ -3219,7 +3215,7 @@
         <v>1.8116883116883118E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.36</v>
       </c>
@@ -3235,7 +3231,7 @@
         <v>1.2077922077922076E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>0.18</v>
       </c>
@@ -3251,7 +3247,7 @@
         <v>6.0389610389610382E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>7.0000000000000007E-2</v>
       </c>

</xml_diff>

<commit_message>
trying only mechanical dispersion as a relation to alpha velocity alpha fits better, alpha is 0.4 to 0.7 cm but in KL/D0 vs Pe plot it is worst, since in y values are similar but in x values are shifted to the left, giving worst physical meaning
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="368" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1BC1358-6400-4665-85E3-F9353679A3E0}"/>
+  <xr:revisionPtr revIDLastSave="379" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7E6D38-8DFC-4BD0-BAFE-F24D09DC2242}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
     <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId10"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_w" sheetId="22" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="24">
   <si>
     <t>KL/D0</t>
   </si>
@@ -114,6 +115,9 @@
   </si>
   <si>
     <t>GomezMendez_etal_2026</t>
+  </si>
+  <si>
+    <t>wGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -432,13 +436,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -446,7 +450,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -454,7 +458,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -462,7 +466,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -470,7 +474,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -478,7 +482,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -486,7 +490,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -494,7 +498,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -502,7 +506,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -510,7 +514,7 @@
         <v>0.435</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -524,7 +528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -532,7 +536,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -548,7 +552,7 @@
         <v>1.9236781609195404</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -564,7 +568,7 @@
         <v>1.7312643678160919</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -580,7 +584,7 @@
         <v>1.5390804597701151</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -596,7 +600,7 @@
         <v>1.3466666666666667</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -612,7 +616,7 @@
         <v>1.1542528735632185</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -628,7 +632,7 @@
         <v>0.96183908045977018</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -644,7 +648,7 @@
         <v>0.76942528735632187</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -660,7 +664,7 @@
         <v>0.57701149425287357</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -676,7 +680,7 @@
         <v>0.38482758620689655</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -692,7 +696,7 @@
         <v>0.19241379310344828</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -708,7 +712,7 @@
         <v>0.14436781609195404</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -724,7 +728,7 @@
         <v>9.6091954022988521E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -748,12 +752,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A19B645C-29D5-4CC1-AB25-EDCCDCB6D159}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -761,7 +765,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -769,7 +773,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -777,7 +781,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -785,7 +789,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -793,7 +797,7 @@
         <v>15.25</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -801,7 +805,7 @@
         <v>0.193</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -809,7 +813,7 @@
         <v>2.6150000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -817,7 +821,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -825,7 +829,7 @@
         <v>0.40720000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -839,7 +843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -847,7 +851,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>0.255637</v>
       </c>
@@ -863,7 +867,7 @@
         <v>1.6416767067779963</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>0.51127500000000003</v>
       </c>
@@ -879,7 +883,7 @@
         <v>3.2833598354616904</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1.2781899000000001</v>
       </c>
@@ -893,6 +897,161 @@
       <c r="D15">
         <f>$B$7*A15/$B$9</f>
         <v>8.2084150012279</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D382D828-8D94-44AF-BFF0-21AA8C62C8CE}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>0.193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.40720000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.255637</v>
+      </c>
+      <c r="B13">
+        <v>1.18</v>
+      </c>
+      <c r="C13">
+        <f>B13/$B$9</f>
+        <v>2.8978388998035363</v>
+      </c>
+      <c r="D13">
+        <f>$B$7*A13/$B$9</f>
+        <v>0.25111689587426328</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.51127500000000003</v>
+      </c>
+      <c r="B14">
+        <v>1.2</v>
+      </c>
+      <c r="C14">
+        <f>B14/$B$9</f>
+        <v>2.9469548133595285</v>
+      </c>
+      <c r="D14">
+        <f>$B$7*A14/$B$9</f>
+        <v>0.50223477406679773</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1.2781899000000001</v>
+      </c>
+      <c r="B15">
+        <v>1.86</v>
+      </c>
+      <c r="C15">
+        <f>B15/$B$9</f>
+        <v>4.5677799607072691</v>
+      </c>
+      <c r="D15">
+        <f>$B$7*A15/$B$9</f>
+        <v>1.255589292730845</v>
       </c>
     </row>
   </sheetData>
@@ -903,13 +1062,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA757B11-61BA-4343-990A-779EA69AE742}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -917,7 +1076,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -925,7 +1084,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -933,7 +1092,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -941,7 +1100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -949,7 +1108,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -957,7 +1116,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -965,7 +1124,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -973,7 +1132,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -981,7 +1140,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -995,7 +1154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1003,7 +1162,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>7.5309999999999997</v>
       </c>
@@ -1019,7 +1178,7 @@
         <v>1.298448275862069</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>6.6950000000000003</v>
       </c>
@@ -1035,7 +1194,7 @@
         <v>1.1543103448275864</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>5.8579999999999997</v>
       </c>
@@ -1051,7 +1210,7 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.0209999999999999</v>
       </c>
@@ -1067,7 +1226,7 @@
         <v>0.86568965517241381</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4.1840000000000002</v>
       </c>
@@ -1083,7 +1242,7 @@
         <v>0.72137931034482772</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3.347</v>
       </c>
@@ -1099,7 +1258,7 @@
         <v>0.57706896551724141</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2.5099999999999998</v>
       </c>
@@ -1115,7 +1274,7 @@
         <v>0.4327586206896552</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -1131,7 +1290,7 @@
         <v>0.2886206896551724</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>0.83699999999999997</v>
       </c>
@@ -1147,7 +1306,7 @@
         <v>0.1443103448275862</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.628</v>
       </c>
@@ -1163,7 +1322,7 @@
         <v>0.10827586206896554</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.41799999999999998</v>
       </c>
@@ -1179,7 +1338,7 @@
         <v>7.2068965517241387E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.20899999999999999</v>
       </c>
@@ -1195,7 +1354,7 @@
         <v>3.6034482758620694E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2.0920000000000001</v>
       </c>
@@ -1219,13 +1378,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4622695-DEB5-4C1F-9455-6739E3C55888}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1233,7 +1392,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1241,7 +1400,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1249,7 +1408,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1257,7 +1416,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1265,7 +1424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1273,7 +1432,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1281,7 +1440,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1289,7 +1448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1297,7 +1456,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1311,7 +1470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1319,7 +1478,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>5.8579999999999997</v>
       </c>
@@ -1335,7 +1494,7 @@
         <v>0.67333333333333334</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>5.0209999999999999</v>
       </c>
@@ -1351,7 +1510,7 @@
         <v>0.57712643678160924</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>4.1840000000000002</v>
       </c>
@@ -1367,7 +1526,7 @@
         <v>0.48091954022988509</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>3.347</v>
       </c>
@@ -1383,7 +1542,7 @@
         <v>0.38471264367816094</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2.9289999999999998</v>
       </c>
@@ -1399,7 +1558,7 @@
         <v>0.33666666666666667</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2.5099999999999998</v>
       </c>
@@ -1415,7 +1574,7 @@
         <v>0.28850574712643678</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2.0920000000000001</v>
       </c>
@@ -1431,7 +1590,7 @@
         <v>0.24045977011494254</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -1447,7 +1606,7 @@
         <v>0.19241379310344828</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.2549999999999999</v>
       </c>
@@ -1463,7 +1622,7 @@
         <v>0.14425287356321839</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -1479,7 +1638,7 @@
         <v>9.6206896551724139E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -1495,7 +1654,7 @@
         <v>7.2183908045977019E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -1511,7 +1670,7 @@
         <v>4.8045977011494261E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -1535,13 +1694,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F522CD30-DFF9-46D4-B41C-E2D69E5568A2}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1549,7 +1708,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1557,7 +1716,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1565,7 +1724,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1573,7 +1732,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1581,7 +1740,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1589,7 +1748,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1597,7 +1756,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1605,7 +1764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1613,7 +1772,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1627,7 +1786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1635,7 +1794,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -1651,7 +1810,7 @@
         <v>1.8112554112554113</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -1667,7 +1826,7 @@
         <v>1.63008658008658</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -1683,7 +1842,7 @@
         <v>1.4491341991341993</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -1699,7 +1858,7 @@
         <v>1.267965367965368</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -1715,7 +1874,7 @@
         <v>1.0867965367965366</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -1731,7 +1890,7 @@
         <v>0.90562770562770567</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -1747,7 +1906,7 @@
         <v>0.72445887445887447</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -1763,7 +1922,7 @@
         <v>0.54329004329004327</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -1779,7 +1938,7 @@
         <v>0.36233766233766229</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -1795,7 +1954,7 @@
         <v>0.18116883116883115</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -1811,7 +1970,7 @@
         <v>0.13593073593073593</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -1827,7 +1986,7 @@
         <v>9.0476190476190474E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -1851,13 +2010,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3833D965-A191-44EF-B626-D5738955DDF0}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1865,7 +2024,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1873,7 +2032,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1881,7 +2040,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1889,7 +2048,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1897,7 +2056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1905,7 +2064,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1913,7 +2072,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1921,7 +2080,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1929,7 +2088,7 @@
         <v>0.61599999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1943,7 +2102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1951,7 +2110,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -1967,7 +2126,7 @@
         <v>1.3584415584415586</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -1983,7 +2142,7 @@
         <v>1.222564935064935</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -1999,7 +2158,7 @@
         <v>1.0868506493506496</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2015,7 +2174,7 @@
         <v>0.95097402597402592</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -2031,7 +2190,7 @@
         <v>0.8150974025974026</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -2047,7 +2206,7 @@
         <v>0.67922077922077928</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -2063,7 +2222,7 @@
         <v>0.54334415584415585</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -2079,7 +2238,7 @@
         <v>0.40746753246753248</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -2095,7 +2254,7 @@
         <v>0.27175324675324675</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -2111,7 +2270,7 @@
         <v>0.13587662337662337</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -2127,7 +2286,7 @@
         <v>0.10194805194805197</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -2143,7 +2302,7 @@
         <v>6.7857142857142866E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -2167,13 +2326,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C470E87-970C-4464-80DC-21CD570DB714}">
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2181,7 +2340,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2189,7 +2348,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2197,7 +2356,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2205,7 +2364,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2213,7 +2372,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2221,7 +2380,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2229,7 +2388,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2237,7 +2396,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2245,7 +2404,7 @@
         <v>0.92400000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2259,7 +2418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2267,7 +2426,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -2283,7 +2442,7 @@
         <v>0.90562770562770567</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -2299,7 +2458,7 @@
         <v>0.81504329004329001</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -2315,7 +2474,7 @@
         <v>0.72456709956709964</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2331,7 +2490,7 @@
         <v>0.63398268398268398</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>5.0209999999999999</v>
       </c>
@@ -2347,7 +2506,7 @@
         <v>0.54339826839826832</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4.1840000000000002</v>
       </c>
@@ -2363,7 +2522,7 @@
         <v>0.45281385281385284</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3.347</v>
       </c>
@@ -2379,7 +2538,7 @@
         <v>0.36222943722943723</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2.5099999999999998</v>
       </c>
@@ -2395,7 +2554,7 @@
         <v>0.27164502164502163</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.6739999999999999</v>
       </c>
@@ -2411,7 +2570,7 @@
         <v>0.18116883116883115</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.83699999999999997</v>
       </c>
@@ -2427,7 +2586,7 @@
         <v>9.0584415584415573E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.628</v>
       </c>
@@ -2443,7 +2602,7 @@
         <v>6.7965367965367965E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.41799999999999998</v>
       </c>
@@ -2459,7 +2618,7 @@
         <v>4.5238095238095237E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.20899999999999999</v>
       </c>
@@ -2483,13 +2642,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC97105-E75A-4887-9BED-937003238E58}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2497,7 +2656,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2505,7 +2664,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2513,7 +2672,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2521,7 +2680,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2529,7 +2688,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2537,7 +2696,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2545,7 +2704,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2553,7 +2712,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2561,7 +2720,7 @@
         <v>0.51200000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2575,7 +2734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2583,7 +2742,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1.85</v>
       </c>
@@ -2599,7 +2758,7 @@
         <v>0.36132812500000006</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>3</v>
       </c>
@@ -2615,7 +2774,7 @@
         <v>0.58593750000000011</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>4.25</v>
       </c>
@@ -2639,13 +2798,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EB6648-E8BE-46BE-A305-6B6827CCA731}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2653,7 +2812,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2661,7 +2820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2669,7 +2828,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2677,7 +2836,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2685,7 +2844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2693,7 +2852,7 @@
         <v>0.10299999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2701,7 +2860,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2709,7 +2868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2717,7 +2876,7 @@
         <v>0.76800000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2731,7 +2890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2739,7 +2898,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8.3680000000000003</v>
       </c>
@@ -2755,7 +2914,7 @@
         <v>1.0895833333333333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>7.5309999999999997</v>
       </c>
@@ -2771,7 +2930,7 @@
         <v>0.98059895833333333</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6.6950000000000003</v>
       </c>
@@ -2787,7 +2946,7 @@
         <v>0.87174479166666674</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5.8579999999999997</v>
       </c>
@@ -2803,7 +2962,7 @@
         <v>0.76276041666666661</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4.1840000000000002</v>
       </c>
@@ -2819,7 +2978,7 @@
         <v>0.54479166666666667</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3.347</v>
       </c>
@@ -2835,7 +2994,7 @@
         <v>0.43580729166666665</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2.5099999999999998</v>
       </c>
@@ -2851,7 +3010,7 @@
         <v>0.32682291666666669</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1.6739999999999999</v>
       </c>
@@ -2867,7 +3026,7 @@
         <v>0.21796874999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>0.83699999999999997</v>
       </c>
@@ -2883,7 +3042,7 @@
         <v>0.10898437499999999</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.628</v>
       </c>
@@ -2899,7 +3058,7 @@
         <v>8.1770833333333348E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.41799999999999998</v>
       </c>
@@ -2915,7 +3074,7 @@
         <v>5.4427083333333334E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.20899999999999999</v>
       </c>
@@ -2939,13 +3098,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316B93C2-C5E9-456C-B87A-12E89A2041DB}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2953,7 +3112,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2961,7 +3120,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2969,7 +3128,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2977,7 +3136,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2985,7 +3144,7 @@
         <v>10.130000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2993,7 +3152,7 @@
         <v>0.20799999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3001,7 +3160,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -3009,7 +3168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -3017,7 +3176,7 @@
         <v>0.92400000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -3031,7 +3190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -3039,7 +3198,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>7.22</v>
       </c>
@@ -3055,7 +3214,7 @@
         <v>0.24222943722943721</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>5.7799999999999994</v>
       </c>
@@ -3071,7 +3230,7 @@
         <v>0.19391774891774888</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>4.33</v>
       </c>
@@ -3087,7 +3246,7 @@
         <v>0.14527056277056274</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>3.61</v>
       </c>
@@ -3103,7 +3262,7 @@
         <v>0.12111471861471861</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2.89</v>
       </c>
@@ -3119,7 +3278,7 @@
         <v>9.6958874458874453E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2.17</v>
       </c>
@@ -3135,7 +3294,7 @@
         <v>7.28030303030303E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1.81</v>
       </c>
@@ -3151,7 +3310,7 @@
         <v>6.0725108225108224E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1.44</v>
       </c>
@@ -3167,7 +3326,7 @@
         <v>4.8311688311688306E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1.08</v>
       </c>
@@ -3183,7 +3342,7 @@
         <v>3.6233766233766236E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>0.72</v>
       </c>
@@ -3199,7 +3358,7 @@
         <v>2.4155844155844153E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>0.54</v>
       </c>
@@ -3215,7 +3374,7 @@
         <v>1.8116883116883118E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.36</v>
       </c>
@@ -3231,7 +3390,7 @@
         <v>1.2077922077922076E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.18</v>
       </c>
@@ -3247,7 +3406,7 @@
         <v>6.0389610389610382E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>7.0000000000000007E-2</v>
       </c>

</xml_diff>

<commit_message>
no mean, results for paper, no good results in log log Kl/D0
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="379" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7E6D38-8DFC-4BD0-BAFE-F24D09DC2242}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D7CAC89-1D1D-41D8-B120-87831B5602D3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
     <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId10"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_w" sheetId="22" r:id="rId11"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500_r" sheetId="23" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -117,7 +117,7 @@
     <t>GomezMendez_etal_2026</t>
   </si>
   <si>
-    <t>wGomezMendez_etal_2026</t>
+    <t>rangeGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -170,6 +170,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -905,7 +909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D382D828-8D94-44AF-BFF0-21AA8C62C8CE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948DB3ED-0929-4F48-9E04-9D67542693A7}">
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -965,7 +969,7 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>0.4</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1011,15 +1015,15 @@
         <v>0.255637</v>
       </c>
       <c r="B13">
-        <v>1.18</v>
+        <v>0.89</v>
       </c>
       <c r="C13">
         <f>B13/$B$9</f>
-        <v>2.8978388998035363</v>
+        <v>2.1856581532416501</v>
       </c>
       <c r="D13">
         <f>$B$7*A13/$B$9</f>
-        <v>0.25111689587426328</v>
+        <v>1.1990831777996069</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1027,15 +1031,15 @@
         <v>0.51127500000000003</v>
       </c>
       <c r="B14">
-        <v>1.2</v>
+        <v>1.31</v>
       </c>
       <c r="C14">
         <f>B14/$B$9</f>
-        <v>2.9469548133595285</v>
+        <v>3.2170923379174852</v>
       </c>
       <c r="D14">
         <f>$B$7*A14/$B$9</f>
-        <v>0.50223477406679773</v>
+        <v>2.3981710461689589</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1043,15 +1047,15 @@
         <v>1.2781899000000001</v>
       </c>
       <c r="B15">
-        <v>1.86</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="C15">
         <f>B15/$B$9</f>
-        <v>4.5677799607072691</v>
+        <v>5.451866404715128</v>
       </c>
       <c r="D15">
         <f>$B$7*A15/$B$9</f>
-        <v>1.255589292730845</v>
+        <v>5.9954388727897845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results for paper after integration all except dabrowski
</commit_message>
<xml_diff>
--- a/input/input_expsAll_results.xlsx
+++ b/input/input_expsAll_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="387" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D7CAC89-1D1D-41D8-B120-87831B5602D3}"/>
+  <xr:revisionPtr revIDLastSave="391" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0256C31-04C4-49AF-A8FF-240BD396AAFA}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kobeissi_FB_H2_CH4_T25_P1450" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,7 @@
     <sheet name="Kobeissi_FB_H2_CO2_T25_P1088" sheetId="8" r:id="rId7"/>
     <sheet name="Kobeissi_FB_H2_CO2_T25_P725" sheetId="9" r:id="rId8"/>
     <sheet name="Yang_BE_H2_N2_T25_P725" sheetId="11" r:id="rId9"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_5" sheetId="21" r:id="rId10"/>
-    <sheet name="GM_BE_H2CO2_T32_P1500_r" sheetId="23" r:id="rId11"/>
+    <sheet name="GM_BE_H2CO2_T32_P1500" sheetId="21" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="23">
   <si>
     <t>KL/D0</t>
   </si>
@@ -115,9 +114,6 @@
   </si>
   <si>
     <t>GomezMendez_etal_2026</t>
-  </si>
-  <si>
-    <t>rangeGomezMendez_etal_2026</t>
   </si>
 </sst>
 </file>
@@ -814,161 +810,6 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>2.6150000000000002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>0.40720000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.255637</v>
-      </c>
-      <c r="B13">
-        <v>1.0456000000000001</v>
-      </c>
-      <c r="C13">
-        <f>B13/$B$9</f>
-        <v>2.5677799607072691</v>
-      </c>
-      <c r="D13">
-        <f>$B$7*A13/$B$9</f>
-        <v>1.6416767067779963</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.51127500000000003</v>
-      </c>
-      <c r="B14">
-        <v>1.4628000000000001</v>
-      </c>
-      <c r="C14">
-        <f>B14/$B$9</f>
-        <v>3.5923379174852652</v>
-      </c>
-      <c r="D14">
-        <f>$B$7*A14/$B$9</f>
-        <v>3.2833598354616904</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1.2781899000000001</v>
-      </c>
-      <c r="B15">
-        <v>2.4708999999999999</v>
-      </c>
-      <c r="C15">
-        <f>B15/$B$9</f>
-        <v>6.0680255402750491</v>
-      </c>
-      <c r="D15">
-        <f>$B$7*A15/$B$9</f>
-        <v>8.2084150012279</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948DB3ED-0929-4F48-9E04-9D67542693A7}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0.193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
         <v>1.91</v>
       </c>
     </row>

</xml_diff>